<commit_message>
Corrrection orth et mise à jour contenus
</commit_message>
<xml_diff>
--- a/documentation/type_contenus.xlsx
+++ b/documentation/type_contenus.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pa.jachiet\prog\exercice_nlp\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F7BBB0D-9B5D-4D5C-8D2D-3EB6B2B7FE7B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2765DB24-6D5E-444D-B359-847F93DCEED0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="103">
   <si>
     <t>Nom du type</t>
   </si>
@@ -344,19 +344,13 @@
     <t>EtudeEtEnquete</t>
   </si>
   <si>
-    <t>non requêtable individuellement ?</t>
-  </si>
-  <si>
     <t>A categoriser</t>
-  </si>
-  <si>
-    <t>Commentaire</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -729,9 +723,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="52.1796875" bestFit="1" customWidth="1"/>
@@ -740,7 +734,7 @@
     <col min="5" max="5" width="34.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -751,13 +745,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>18</v>
       </c>
@@ -771,7 +762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>57</v>
       </c>
@@ -782,7 +773,7 @@
         <v>6323</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -793,7 +784,7 @@
         <v>6155</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -804,7 +795,7 @@
         <v>4498</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>61</v>
       </c>
@@ -815,7 +806,7 @@
         <v>3727</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -829,7 +820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>85</v>
       </c>
@@ -840,7 +831,7 @@
         <v>3282</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>37</v>
       </c>
@@ -851,7 +842,7 @@
         <v>1501</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>53</v>
       </c>
@@ -862,7 +853,7 @@
         <v>1164</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -873,7 +864,7 @@
         <v>1074</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
@@ -884,7 +875,7 @@
         <v>1035</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>94</v>
       </c>
@@ -894,14 +885,8 @@
       <c r="C13">
         <v>621</v>
       </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>35</v>
       </c>
@@ -915,7 +900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>75</v>
       </c>
@@ -929,7 +914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>66</v>
       </c>
@@ -940,7 +925,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>68</v>
       </c>
@@ -949,6 +934,9 @@
       </c>
       <c r="C17">
         <v>317</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -976,7 +964,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>48</v>
       </c>
@@ -985,6 +973,9 @@
       </c>
       <c r="C20">
         <v>176</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
@@ -1045,7 +1036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>100</v>
       </c>
@@ -1054,6 +1045,9 @@
       </c>
       <c r="C26">
         <v>109</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
@@ -1371,7 +1365,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E54">
+  <autoFilter ref="A1:E54" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="3">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>

</xml_diff>